<commit_message>
docs: record V61 public verification and final workbook
</commit_message>
<xml_diff>
--- a/docs/THE_PIT_STAGES_V61_SUIVI.xlsx
+++ b/docs/THE_PIT_STAGES_V61_SUIVI.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AnimationsV61" sheetId="1" r:id="Ree52c248cf934a5b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resteclasseur" sheetId="2" r:id="R010f3881f11f4178"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AnimationsV61" sheetId="1" r:id="R29cfad8ffa0a47e4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resteclasseur" sheetId="2" r:id="R74e8e9fd4f7c4940"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -17,7 +17,7 @@
   <x:numFmts count="1">
     <x:numFmt numFmtId="200" formatCode="0"/>
   </x:numFmts>
-  <x:fonts count="5">
+  <x:fonts count="6">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -31,6 +31,11 @@
       <x:b/>
       <x:sz val="14"/>
       <x:color rgb="FF172834"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:sz val="9"/>
+      <x:color rgb="FF465863"/>
       <x:name val="Arial"/>
     </x:font>
     <x:font>
@@ -70,7 +75,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="18">
+  <x:cellXfs count="20">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -97,22 +102,28 @@
     <x:xf numFmtId="200" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="top" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="0"/>
+    </x:xf>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="top" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="200" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="200" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -472,8 +483,10 @@
       <x:c r="J6" s="3"/>
       <x:c r="K6" s="3"/>
     </x:row>
-    <x:row r="7">
-      <x:c r="A7" s="3"/>
+    <x:row r="7" ht="20" customHeight="1">
+      <x:c r="A7" s="11" t="str">
+        <x:v>Publication contrôlée : https://yautja-la-longue-chasse.vercel.app — commit c9feb1d0ae4f514ee737380eb786543b00039845</x:v>
+      </x:c>
       <x:c r="B7" s="3"/>
       <x:c r="C7" s="3"/>
       <x:c r="D7" s="3"/>
@@ -486,40 +499,40 @@
       <x:c r="K7" s="3"/>
     </x:row>
     <x:row r="8" ht="36" customHeight="1">
-      <x:c r="A8" s="13" t="str">
+      <x:c r="A8" s="15" t="str">
         <x:v>Scène</x:v>
       </x:c>
-      <x:c r="B8" s="13" t="str">
+      <x:c r="B8" s="15" t="str">
         <x:v>Arène</x:v>
       </x:c>
-      <x:c r="C8" s="13" t="str">
+      <x:c r="C8" s="15" t="str">
         <x:v>Animation</x:v>
       </x:c>
-      <x:c r="D8" s="13" t="str">
+      <x:c r="D8" s="15" t="str">
         <x:v>Dessins</x:v>
       </x:c>
-      <x:c r="E8" s="13" t="str">
+      <x:c r="E8" s="15" t="str">
         <x:v>Origine</x:v>
       </x:c>
-      <x:c r="F8" s="13" t="str">
+      <x:c r="F8" s="15" t="str">
         <x:v>Déclenchement</x:v>
       </x:c>
-      <x:c r="G8" s="13" t="str">
+      <x:c r="G8" s="15" t="str">
         <x:v>Contrôle du jeu</x:v>
       </x:c>
-      <x:c r="H8" s="13" t="str">
+      <x:c r="H8" s="15" t="str">
         <x:v>Limites et conditions</x:v>
       </x:c>
-      <x:c r="I8" s="13" t="str">
+      <x:c r="I8" s="15" t="str">
         <x:v>Publication</x:v>
       </x:c>
-      <x:c r="J8" s="17" t="str"/>
-      <x:c r="K8" s="15" t="str">
+      <x:c r="J8" s="19" t="str"/>
+      <x:c r="K8" s="17" t="str">
         <x:v>Sources par animation</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="54" customHeight="1">
-      <x:c r="A9" s="16" t="n">
+      <x:c r="A9" s="18" t="n">
         <x:v>139</x:v>
       </x:c>
       <x:c r="B9" s="3" t="str">
@@ -528,7 +541,7 @@
       <x:c r="C9" s="3" t="str">
         <x:v>Hélicoptère de police lointain — rotor</x:v>
       </x:c>
-      <x:c r="D9" s="16" t="n">
+      <x:c r="D9" s="18" t="n">
         <x:v>6</x:v>
       </x:c>
       <x:c r="E9" s="3" t="str">
@@ -544,9 +557,9 @@
         <x:v>Toits et véhicules originaux adaptés à Gotham. Aucun modèle exact ou policier nommé certifié.</x:v>
       </x:c>
       <x:c r="I9" s="3" t="str">
-        <x:v>Publication non vérifiée</x:v>
-      </x:c>
-      <x:c r="J9" s="17"/>
+        <x:v>Publié, lot contrôlé</x:v>
+      </x:c>
+      <x:c r="J9" s="19"/>
       <x:c r="K9" s="3" t="str">
         <x:v>139 — Hélicoptère de police lointain — rotor
 10_VIE_DES_STAGES!E92
@@ -554,7 +567,7 @@
       </x:c>
     </x:row>
     <x:row r="10" ht="54" customHeight="1">
-      <x:c r="A10" s="16" t="n">
+      <x:c r="A10" s="18" t="n">
         <x:v>139</x:v>
       </x:c>
       <x:c r="B10" s="3" t="str">
@@ -563,7 +576,7 @@
       <x:c r="C10" s="3" t="str">
         <x:v>Policier anonyme — veille et radio</x:v>
       </x:c>
-      <x:c r="D10" s="16" t="n">
+      <x:c r="D10" s="18" t="n">
         <x:v>6</x:v>
       </x:c>
       <x:c r="E10" s="3" t="str">
@@ -579,9 +592,9 @@
         <x:v>Toits et véhicules originaux adaptés à Gotham. Aucun modèle exact ou policier nommé certifié.</x:v>
       </x:c>
       <x:c r="I10" s="3" t="str">
-        <x:v>Publication non vérifiée</x:v>
-      </x:c>
-      <x:c r="J10" s="17"/>
+        <x:v>Publié, lot contrôlé</x:v>
+      </x:c>
+      <x:c r="J10" s="19"/>
       <x:c r="K10" s="3" t="str">
         <x:v>139 — Policier anonyme — veille et radio
 10_VIE_DES_STAGES!E93
@@ -589,7 +602,7 @@
       </x:c>
     </x:row>
     <x:row r="11" ht="54" customHeight="1">
-      <x:c r="A11" s="16" t="n">
+      <x:c r="A11" s="18" t="n">
         <x:v>139</x:v>
       </x:c>
       <x:c r="B11" s="3" t="str">
@@ -598,7 +611,7 @@
       <x:c r="C11" s="3" t="str">
         <x:v>Gargouille — linge au vent</x:v>
       </x:c>
-      <x:c r="D11" s="16" t="n">
+      <x:c r="D11" s="18" t="n">
         <x:v>6</x:v>
       </x:c>
       <x:c r="E11" s="3" t="str">
@@ -614,9 +627,9 @@
         <x:v>Toits et véhicules originaux adaptés à Gotham. Aucun modèle exact ou policier nommé certifié.</x:v>
       </x:c>
       <x:c r="I11" s="3" t="str">
-        <x:v>Publication non vérifiée</x:v>
-      </x:c>
-      <x:c r="J11" s="17"/>
+        <x:v>Publié, lot contrôlé</x:v>
+      </x:c>
+      <x:c r="J11" s="19"/>
       <x:c r="K11" s="3" t="str">
         <x:v>139 — Gargouille — linge au vent
 10_VIE_DES_STAGES!E94
@@ -624,7 +637,7 @@
       </x:c>
     </x:row>
     <x:row r="12" ht="54" customHeight="1">
-      <x:c r="A12" s="16" t="n">
+      <x:c r="A12" s="18" t="n">
         <x:v>140</x:v>
       </x:c>
       <x:c r="B12" s="3" t="str">
@@ -633,7 +646,7 @@
       <x:c r="C12" s="3" t="str">
         <x:v>Papillons nocturnes sur un rameau de pin</x:v>
       </x:c>
-      <x:c r="D12" s="16" t="n">
+      <x:c r="D12" s="18" t="n">
         <x:v>6</x:v>
       </x:c>
       <x:c r="E12" s="3" t="str">
@@ -649,9 +662,9 @@
         <x:v>Garde anonyme seulement après le duel. Aucun Enforcer nommé ou lien biographique de Skinner inventé.</x:v>
       </x:c>
       <x:c r="I12" s="3" t="str">
-        <x:v>Publication non vérifiée</x:v>
-      </x:c>
-      <x:c r="J12" s="17"/>
+        <x:v>Publié, lot contrôlé</x:v>
+      </x:c>
+      <x:c r="J12" s="19"/>
       <x:c r="K12" s="3" t="str">
         <x:v>140 — Papillons nocturnes sur un rameau de pin
 10_VIE_DES_STAGES!E71
@@ -659,7 +672,7 @@
       </x:c>
     </x:row>
     <x:row r="13" ht="54" customHeight="1">
-      <x:c r="A13" s="16" t="n">
+      <x:c r="A13" s="18" t="n">
         <x:v>140</x:v>
       </x:c>
       <x:c r="B13" s="3" t="str">
@@ -668,7 +681,7 @@
       <x:c r="C13" s="3" t="str">
         <x:v>Broussailles frôlées par une proie hors champ</x:v>
       </x:c>
-      <x:c r="D13" s="16" t="n">
+      <x:c r="D13" s="18" t="n">
         <x:v>6</x:v>
       </x:c>
       <x:c r="E13" s="3" t="str">
@@ -684,9 +697,9 @@
         <x:v>Garde anonyme seulement après le duel. Aucun Enforcer nommé ou lien biographique de Skinner inventé.</x:v>
       </x:c>
       <x:c r="I13" s="3" t="str">
-        <x:v>Publication non vérifiée</x:v>
-      </x:c>
-      <x:c r="J13" s="17"/>
+        <x:v>Publié, lot contrôlé</x:v>
+      </x:c>
+      <x:c r="J13" s="19"/>
       <x:c r="K13" s="3" t="str">
         <x:v>140 — Broussailles frôlées par une proie hors champ
 10_VIE_DES_STAGES!E72
@@ -694,7 +707,7 @@
       </x:c>
     </x:row>
     <x:row r="14" ht="54" customHeight="1">
-      <x:c r="A14" s="16" t="n">
+      <x:c r="A14" s="18" t="n">
         <x:v>140</x:v>
       </x:c>
       <x:c r="B14" s="3" t="str">
@@ -703,7 +716,7 @@
       <x:c r="C14" s="3" t="str">
         <x:v>Balise mécanique originale — fumée résiduelle</x:v>
       </x:c>
-      <x:c r="D14" s="16" t="n">
+      <x:c r="D14" s="18" t="n">
         <x:v>6</x:v>
       </x:c>
       <x:c r="E14" s="3" t="str">
@@ -719,9 +732,9 @@
         <x:v>Garde anonyme seulement après le duel. Aucun Enforcer nommé ou lien biographique de Skinner inventé.</x:v>
       </x:c>
       <x:c r="I14" s="3" t="str">
-        <x:v>Publication non vérifiée</x:v>
-      </x:c>
-      <x:c r="J14" s="17"/>
+        <x:v>Publié, lot contrôlé</x:v>
+      </x:c>
+      <x:c r="J14" s="19"/>
       <x:c r="K14" s="3" t="str">
         <x:v>140 — Balise mécanique originale — fumée résiduelle
 10_VIE_DES_STAGES!E73
@@ -729,7 +742,7 @@
       </x:c>
     </x:row>
     <x:row r="15" ht="54" customHeight="1">
-      <x:c r="A15" s="16" t="n">
+      <x:c r="A15" s="18" t="n">
         <x:v>140</x:v>
       </x:c>
       <x:c r="B15" s="3" t="str">
@@ -738,7 +751,7 @@
       <x:c r="C15" s="3" t="str">
         <x:v>Garde anonyme — observation après le duel</x:v>
       </x:c>
-      <x:c r="D15" s="16" t="n">
+      <x:c r="D15" s="18" t="n">
         <x:v>6</x:v>
       </x:c>
       <x:c r="E15" s="3" t="str">
@@ -754,9 +767,9 @@
         <x:v>Garde anonyme seulement après le duel. Aucun Enforcer nommé ou lien biographique de Skinner inventé.</x:v>
       </x:c>
       <x:c r="I15" s="3" t="str">
-        <x:v>Publication non vérifiée</x:v>
-      </x:c>
-      <x:c r="J15" s="17"/>
+        <x:v>Publié, lot contrôlé</x:v>
+      </x:c>
+      <x:c r="J15" s="19"/>
       <x:c r="K15" s="3" t="str">
         <x:v>140 — Garde anonyme — observation après le duel
 10_VIE_DES_STAGES!E71
@@ -764,7 +777,7 @@
       </x:c>
     </x:row>
     <x:row r="16" ht="54" customHeight="1">
-      <x:c r="A16" s="16" t="n">
+      <x:c r="A16" s="18" t="n">
         <x:v>142</x:v>
       </x:c>
       <x:c r="B16" s="3" t="str">
@@ -773,7 +786,7 @@
       <x:c r="C16" s="3" t="str">
         <x:v>Ombre de xénomorphe — mouvement sur la brique</x:v>
       </x:c>
-      <x:c r="D16" s="16" t="n">
+      <x:c r="D16" s="18" t="n">
         <x:v>6</x:v>
       </x:c>
       <x:c r="E16" s="3" t="str">
@@ -789,9 +802,9 @@
         <x:v>Adaptation du fan-film Dead End. Patrouille anonyme conditionnée à la fin du duel, sans identité canonique inventée.</x:v>
       </x:c>
       <x:c r="I16" s="3" t="str">
-        <x:v>Publication non vérifiée</x:v>
-      </x:c>
-      <x:c r="J16" s="17"/>
+        <x:v>Publié, lot contrôlé</x:v>
+      </x:c>
+      <x:c r="J16" s="19"/>
       <x:c r="K16" s="3" t="str">
         <x:v>142 — Ombre de xénomorphe — mouvement sur la brique
 10_VIE_DES_STAGES!E110
@@ -799,7 +812,7 @@
       </x:c>
     </x:row>
     <x:row r="17" ht="54" customHeight="1">
-      <x:c r="A17" s="16" t="n">
+      <x:c r="A17" s="18" t="n">
         <x:v>142</x:v>
       </x:c>
       <x:c r="B17" s="3" t="str">
@@ -808,7 +821,7 @@
       <x:c r="C17" s="3" t="str">
         <x:v>Ventilation murale — vapeur et gouttes</x:v>
       </x:c>
-      <x:c r="D17" s="16" t="n">
+      <x:c r="D17" s="18" t="n">
         <x:v>6</x:v>
       </x:c>
       <x:c r="E17" s="3" t="str">
@@ -824,9 +837,9 @@
         <x:v>Adaptation du fan-film Dead End. Patrouille anonyme conditionnée à la fin du duel, sans identité canonique inventée.</x:v>
       </x:c>
       <x:c r="I17" s="3" t="str">
-        <x:v>Publication non vérifiée</x:v>
-      </x:c>
-      <x:c r="J17" s="17"/>
+        <x:v>Publié, lot contrôlé</x:v>
+      </x:c>
+      <x:c r="J17" s="19"/>
       <x:c r="K17" s="3" t="str">
         <x:v>142 — Ventilation murale — vapeur et gouttes
 10_VIE_DES_STAGES!E111
@@ -834,7 +847,7 @@
       </x:c>
     </x:row>
     <x:row r="18" ht="54" customHeight="1">
-      <x:c r="A18" s="16" t="n">
+      <x:c r="A18" s="18" t="n">
         <x:v>142</x:v>
       </x:c>
       <x:c r="B18" s="3" t="str">
@@ -843,7 +856,7 @@
       <x:c r="C18" s="3" t="str">
         <x:v>Câble et tissu — souffle de la ruelle</x:v>
       </x:c>
-      <x:c r="D18" s="16" t="n">
+      <x:c r="D18" s="18" t="n">
         <x:v>6</x:v>
       </x:c>
       <x:c r="E18" s="3" t="str">
@@ -859,9 +872,9 @@
         <x:v>Adaptation du fan-film Dead End. Patrouille anonyme conditionnée à la fin du duel, sans identité canonique inventée.</x:v>
       </x:c>
       <x:c r="I18" s="3" t="str">
-        <x:v>Publication non vérifiée</x:v>
-      </x:c>
-      <x:c r="J18" s="17"/>
+        <x:v>Publié, lot contrôlé</x:v>
+      </x:c>
+      <x:c r="J18" s="19"/>
       <x:c r="K18" s="3" t="str">
         <x:v>142 — Câble et tissu — souffle de la ruelle
 10_VIE_DES_STAGES!E112
@@ -869,7 +882,7 @@
       </x:c>
     </x:row>
     <x:row r="19" ht="54" customHeight="1">
-      <x:c r="A19" s="16" t="n">
+      <x:c r="A19" s="18" t="n">
         <x:v>142</x:v>
       </x:c>
       <x:c r="B19" s="3" t="str">
@@ -878,7 +891,7 @@
       <x:c r="C19" s="3" t="str">
         <x:v>Deux chasseurs anonymes — relève après le duel</x:v>
       </x:c>
-      <x:c r="D19" s="16" t="n">
+      <x:c r="D19" s="18" t="n">
         <x:v>6</x:v>
       </x:c>
       <x:c r="E19" s="3" t="str">
@@ -894,9 +907,9 @@
         <x:v>Adaptation du fan-film Dead End. Patrouille anonyme conditionnée à la fin du duel, sans identité canonique inventée.</x:v>
       </x:c>
       <x:c r="I19" s="3" t="str">
-        <x:v>Publication non vérifiée</x:v>
-      </x:c>
-      <x:c r="J19" s="17"/>
+        <x:v>Publié, lot contrôlé</x:v>
+      </x:c>
+      <x:c r="J19" s="19"/>
       <x:c r="K19" s="3" t="str">
         <x:v>142 — Deux chasseurs anonymes — relève après le duel
 10_VIE_DES_STAGES!E112
@@ -904,7 +917,7 @@
       </x:c>
     </x:row>
     <x:row r="20" ht="76.5" customHeight="1">
-      <x:c r="A20" s="16" t="n">
+      <x:c r="A20" s="18" t="n">
         <x:v>144</x:v>
       </x:c>
       <x:c r="B20" s="3" t="str">
@@ -913,7 +926,7 @@
       <x:c r="C20" s="3" t="str">
         <x:v>Enseigne du diner — tissu et chaînes</x:v>
       </x:c>
-      <x:c r="D20" s="16" t="n">
+      <x:c r="D20" s="18" t="n">
         <x:v>6</x:v>
       </x:c>
       <x:c r="E20" s="3" t="str">
@@ -929,9 +942,9 @@
         <x:v>Adultes originaux uniquement. Course dans une ouverture arrière, masquée au repos et en mouvement réduit.</x:v>
       </x:c>
       <x:c r="I20" s="3" t="str">
-        <x:v>Publication non vérifiée</x:v>
-      </x:c>
-      <x:c r="J20" s="17"/>
+        <x:v>Publié, lot contrôlé</x:v>
+      </x:c>
+      <x:c r="J20" s="19"/>
       <x:c r="K20" s="3" t="str">
         <x:v>144 — Enseigne du diner — tissu et chaînes
 10_VIE_DES_STAGES!E101
@@ -940,7 +953,7 @@
       </x:c>
     </x:row>
     <x:row r="21" ht="76.5" customHeight="1">
-      <x:c r="A21" s="16" t="n">
+      <x:c r="A21" s="18" t="n">
         <x:v>144</x:v>
       </x:c>
       <x:c r="B21" s="3" t="str">
@@ -949,7 +962,7 @@
       <x:c r="C21" s="3" t="str">
         <x:v>Ambulance anonyme — suspension et roues</x:v>
       </x:c>
-      <x:c r="D21" s="16" t="n">
+      <x:c r="D21" s="18" t="n">
         <x:v>6</x:v>
       </x:c>
       <x:c r="E21" s="3" t="str">
@@ -965,9 +978,9 @@
         <x:v>Adultes originaux uniquement. Course dans une ouverture arrière, masquée au repos et en mouvement réduit.</x:v>
       </x:c>
       <x:c r="I21" s="3" t="str">
-        <x:v>Publication non vérifiée</x:v>
-      </x:c>
-      <x:c r="J21" s="17"/>
+        <x:v>Publié, lot contrôlé</x:v>
+      </x:c>
+      <x:c r="J21" s="19"/>
       <x:c r="K21" s="3" t="str">
         <x:v>144 — Ambulance anonyme — suspension et roues
 10_VIE_DES_STAGES!E102
@@ -976,7 +989,7 @@
       </x:c>
     </x:row>
     <x:row r="22" ht="76.5" customHeight="1">
-      <x:c r="A22" s="16" t="n">
+      <x:c r="A22" s="18" t="n">
         <x:v>144</x:v>
       </x:c>
       <x:c r="B22" s="3" t="str">
@@ -985,7 +998,7 @@
       <x:c r="C22" s="3" t="str">
         <x:v>Habitants adultes — fuite derrière la vitrine</x:v>
       </x:c>
-      <x:c r="D22" s="16" t="n">
+      <x:c r="D22" s="18" t="n">
         <x:v>6</x:v>
       </x:c>
       <x:c r="E22" s="3" t="str">
@@ -1001,9 +1014,9 @@
         <x:v>Adultes originaux uniquement. Course dans une ouverture arrière, masquée au repos et en mouvement réduit.</x:v>
       </x:c>
       <x:c r="I22" s="3" t="str">
-        <x:v>Publication non vérifiée</x:v>
-      </x:c>
-      <x:c r="J22" s="17"/>
+        <x:v>Publié, lot contrôlé</x:v>
+      </x:c>
+      <x:c r="J22" s="19"/>
       <x:c r="K22" s="3" t="str">
         <x:v>144 — Habitants adultes — fuite derrière la vitrine
 10_VIE_DES_STAGES!E103
@@ -1012,7 +1025,7 @@
       </x:c>
     </x:row>
     <x:row r="23" ht="54" customHeight="1">
-      <x:c r="A23" s="16" t="n">
+      <x:c r="A23" s="18" t="n">
         <x:v>146</x:v>
       </x:c>
       <x:c r="B23" s="3" t="str">
@@ -1021,7 +1034,7 @@
       <x:c r="C23" s="3" t="str">
         <x:v>Dais ancien — colliers mécaniques</x:v>
       </x:c>
-      <x:c r="D23" s="16" t="n">
+      <x:c r="D23" s="18" t="n">
         <x:v>6</x:v>
       </x:c>
       <x:c r="E23" s="3" t="str">
@@ -1037,9 +1050,9 @@
         <x:v>Mécanisme et poussière adaptés. Apparence exacte de la faune non vérifiée : végétation de remplacement déclarée.</x:v>
       </x:c>
       <x:c r="I23" s="3" t="str">
-        <x:v>Publication non vérifiée</x:v>
-      </x:c>
-      <x:c r="J23" s="17"/>
+        <x:v>Publié, lot contrôlé</x:v>
+      </x:c>
+      <x:c r="J23" s="19"/>
       <x:c r="K23" s="3" t="str">
         <x:v>146 — Dais ancien — colliers mécaniques
 10_VIE_DES_STAGES!E146
@@ -1047,7 +1060,7 @@
       </x:c>
     </x:row>
     <x:row r="24" ht="48" customHeight="1">
-      <x:c r="A24" s="16" t="n">
+      <x:c r="A24" s="18" t="n">
         <x:v>146</x:v>
       </x:c>
       <x:c r="B24" s="3" t="str">
@@ -1056,7 +1069,7 @@
       <x:c r="C24" s="3" t="str">
         <x:v>Fougères sur corniche — souffle humide</x:v>
       </x:c>
-      <x:c r="D24" s="16" t="n">
+      <x:c r="D24" s="18" t="n">
         <x:v>6</x:v>
       </x:c>
       <x:c r="E24" s="3" t="str">
@@ -1072,16 +1085,16 @@
         <x:v>Mécanisme et poussière adaptés. Apparence exacte de la faune non vérifiée : végétation de remplacement déclarée.</x:v>
       </x:c>
       <x:c r="I24" s="3" t="str">
-        <x:v>Publication non vérifiée</x:v>
-      </x:c>
-      <x:c r="J24" s="17"/>
+        <x:v>Publié, lot contrôlé</x:v>
+      </x:c>
+      <x:c r="J24" s="19"/>
       <x:c r="K24" s="3" t="str">
         <x:v>146 — Fougères sur corniche — souffle humide
 10_VIE_DES_STAGES!E147</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="48" customHeight="1">
-      <x:c r="A25" s="16" t="n">
+      <x:c r="A25" s="18" t="n">
         <x:v>146</x:v>
       </x:c>
       <x:c r="B25" s="3" t="str">
@@ -1090,7 +1103,7 @@
       <x:c r="C25" s="3" t="str">
         <x:v>Porte de pierre — iris et poussière</x:v>
       </x:c>
-      <x:c r="D25" s="16" t="n">
+      <x:c r="D25" s="18" t="n">
         <x:v>6</x:v>
       </x:c>
       <x:c r="E25" s="3" t="str">
@@ -1106,16 +1119,16 @@
         <x:v>Mécanisme et poussière adaptés. Apparence exacte de la faune non vérifiée : végétation de remplacement déclarée.</x:v>
       </x:c>
       <x:c r="I25" s="3" t="str">
-        <x:v>Publication non vérifiée</x:v>
-      </x:c>
-      <x:c r="J25" s="17"/>
+        <x:v>Publié, lot contrôlé</x:v>
+      </x:c>
+      <x:c r="J25" s="19"/>
       <x:c r="K25" s="3" t="str">
         <x:v>146 — Porte de pierre — iris et poussière
 10_VIE_DES_STAGES!E148</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="87.75" customHeight="1">
-      <x:c r="A26" s="16" t="n">
+      <x:c r="A26" s="18" t="n">
         <x:v>155</x:v>
       </x:c>
       <x:c r="B26" s="3" t="str">
@@ -1124,7 +1137,7 @@
       <x:c r="C26" s="3" t="str">
         <x:v>Judge anonyme — patrouille et radio</x:v>
       </x:c>
-      <x:c r="D26" s="16" t="n">
+      <x:c r="D26" s="18" t="n">
         <x:v>6</x:v>
       </x:c>
       <x:c r="E26" s="3" t="str">
@@ -1140,9 +1153,9 @@
         <x:v>Mega-City One adaptée. Costume et véhicules à lire selon les limites des sources inspectées.</x:v>
       </x:c>
       <x:c r="I26" s="3" t="str">
-        <x:v>Publication non vérifiée</x:v>
-      </x:c>
-      <x:c r="J26" s="17"/>
+        <x:v>Publié, lot contrôlé</x:v>
+      </x:c>
+      <x:c r="J26" s="19"/>
       <x:c r="K26" s="3" t="str">
         <x:v>155 — Judge anonyme — patrouille et radio
 10_VIE_DES_STAGES!E98
@@ -1151,7 +1164,7 @@
       </x:c>
     </x:row>
     <x:row r="27" ht="87.75" customHeight="1">
-      <x:c r="A27" s="16" t="n">
+      <x:c r="A27" s="18" t="n">
         <x:v>155</x:v>
       </x:c>
       <x:c r="B27" s="3" t="str">
@@ -1160,7 +1173,7 @@
       <x:c r="C27" s="3" t="str">
         <x:v>Transport aérien original — stabilisateurs</x:v>
       </x:c>
-      <x:c r="D27" s="16" t="n">
+      <x:c r="D27" s="18" t="n">
         <x:v>6</x:v>
       </x:c>
       <x:c r="E27" s="3" t="str">
@@ -1176,9 +1189,9 @@
         <x:v>Mega-City One adaptée. Costume et véhicules à lire selon les limites des sources inspectées.</x:v>
       </x:c>
       <x:c r="I27" s="3" t="str">
-        <x:v>Publication non vérifiée</x:v>
-      </x:c>
-      <x:c r="J27" s="17"/>
+        <x:v>Publié, lot contrôlé</x:v>
+      </x:c>
+      <x:c r="J27" s="19"/>
       <x:c r="K27" s="3" t="str">
         <x:v>155 — Transport aérien original — stabilisateurs
 10_VIE_DES_STAGES!E99
@@ -1187,7 +1200,7 @@
       </x:c>
     </x:row>
     <x:row r="28" ht="87.75" customHeight="1">
-      <x:c r="A28" s="16" t="n">
+      <x:c r="A28" s="18" t="n">
         <x:v>155</x:v>
       </x:c>
       <x:c r="B28" s="3" t="str">
@@ -1196,7 +1209,7 @@
       <x:c r="C28" s="3" t="str">
         <x:v>Écran municipal — réseau de transport</x:v>
       </x:c>
-      <x:c r="D28" s="16" t="n">
+      <x:c r="D28" s="18" t="n">
         <x:v>6</x:v>
       </x:c>
       <x:c r="E28" s="3" t="str">
@@ -1212,9 +1225,9 @@
         <x:v>Mega-City One adaptée. Costume et véhicules à lire selon les limites des sources inspectées.</x:v>
       </x:c>
       <x:c r="I28" s="3" t="str">
-        <x:v>Publication non vérifiée</x:v>
-      </x:c>
-      <x:c r="J28" s="17"/>
+        <x:v>Publié, lot contrôlé</x:v>
+      </x:c>
+      <x:c r="J28" s="19"/>
       <x:c r="K28" s="3" t="str">
         <x:v>155 — Écran municipal — réseau de transport
 10_VIE_DES_STAGES!E100
@@ -1223,7 +1236,7 @@
       </x:c>
     </x:row>
     <x:row r="29" ht="65.25" customHeight="1">
-      <x:c r="A29" s="16" t="n">
+      <x:c r="A29" s="18" t="n">
         <x:v>156</x:v>
       </x:c>
       <x:c r="B29" s="3" t="str">
@@ -1232,7 +1245,7 @@
       <x:c r="C29" s="3" t="str">
         <x:v>Construction jaune originale — panneaux mobiles</x:v>
       </x:c>
-      <x:c r="D29" s="16" t="n">
+      <x:c r="D29" s="18" t="n">
         <x:v>6</x:v>
       </x:c>
       <x:c r="E29" s="3" t="str">
@@ -1248,9 +1261,9 @@
         <x:v>Terrasse terrestre originale. Visiteurs non validés absents. Géométrie non reproduite depuis une planche exacte.</x:v>
       </x:c>
       <x:c r="I29" s="3" t="str">
-        <x:v>Publication non vérifiée</x:v>
-      </x:c>
-      <x:c r="J29" s="17"/>
+        <x:v>Publié, lot contrôlé</x:v>
+      </x:c>
+      <x:c r="J29" s="19"/>
       <x:c r="K29" s="3" t="str">
         <x:v>156 — Construction jaune originale — panneaux mobiles
 10_VIE_DES_STAGES!E107
@@ -1259,7 +1272,7 @@
       </x:c>
     </x:row>
     <x:row r="30" ht="65.25" customHeight="1">
-      <x:c r="A30" s="16" t="n">
+      <x:c r="A30" s="18" t="n">
         <x:v>156</x:v>
       </x:c>
       <x:c r="B30" s="3" t="str">
@@ -1268,7 +1281,7 @@
       <x:c r="C30" s="3" t="str">
         <x:v>Extracteur de toiture — rotation des ailettes</x:v>
       </x:c>
-      <x:c r="D30" s="16" t="n">
+      <x:c r="D30" s="18" t="n">
         <x:v>6</x:v>
       </x:c>
       <x:c r="E30" s="3" t="str">
@@ -1284,9 +1297,9 @@
         <x:v>Terrasse terrestre originale. Visiteurs non validés absents. Géométrie non reproduite depuis une planche exacte.</x:v>
       </x:c>
       <x:c r="I30" s="3" t="str">
-        <x:v>Publication non vérifiée</x:v>
-      </x:c>
-      <x:c r="J30" s="17"/>
+        <x:v>Publié, lot contrôlé</x:v>
+      </x:c>
+      <x:c r="J30" s="19"/>
       <x:c r="K30" s="3" t="str">
         <x:v>156 — Extracteur de toiture — rotation des ailettes
 10_VIE_DES_STAGES!E108
@@ -1295,7 +1308,7 @@
       </x:c>
     </x:row>
     <x:row r="31" ht="65.25" customHeight="1">
-      <x:c r="A31" s="16" t="n">
+      <x:c r="A31" s="18" t="n">
         <x:v>156</x:v>
       </x:c>
       <x:c r="B31" s="3" t="str">
@@ -1304,7 +1317,7 @@
       <x:c r="C31" s="3" t="str">
         <x:v>Halo jaune stable — particules orbitales</x:v>
       </x:c>
-      <x:c r="D31" s="16" t="n">
+      <x:c r="D31" s="18" t="n">
         <x:v>6</x:v>
       </x:c>
       <x:c r="E31" s="3" t="str">
@@ -1320,9 +1333,9 @@
         <x:v>Terrasse terrestre originale. Visiteurs non validés absents. Géométrie non reproduite depuis une planche exacte.</x:v>
       </x:c>
       <x:c r="I31" s="3" t="str">
-        <x:v>Publication non vérifiée</x:v>
-      </x:c>
-      <x:c r="J31" s="17"/>
+        <x:v>Publié, lot contrôlé</x:v>
+      </x:c>
+      <x:c r="J31" s="19"/>
       <x:c r="K31" s="3" t="str">
         <x:v>156 — Halo jaune stable — particules orbitales
 10_VIE_DES_STAGES!E109
@@ -1331,7 +1344,7 @@
       </x:c>
     </x:row>
     <x:row r="32" ht="48" customHeight="1">
-      <x:c r="A32" s="16" t="n">
+      <x:c r="A32" s="18" t="n">
         <x:v>165</x:v>
       </x:c>
       <x:c r="B32" s="3" t="str">
@@ -1340,7 +1353,7 @@
       <x:c r="C32" s="3" t="str">
         <x:v>Garde anonyme — salut de victoire</x:v>
       </x:c>
-      <x:c r="D32" s="16" t="n">
+      <x:c r="D32" s="18" t="n">
         <x:v>6</x:v>
       </x:c>
       <x:c r="E32" s="3" t="str">
@@ -1356,16 +1369,16 @@
         <x:v>Salut d’un garde anonyme lié au résultat. Aucun dirigeant nommé ou tentacule ajouté.</x:v>
       </x:c>
       <x:c r="I32" s="3" t="str">
-        <x:v>Publication non vérifiée</x:v>
-      </x:c>
-      <x:c r="J32" s="17"/>
+        <x:v>Publié, lot contrôlé</x:v>
+      </x:c>
+      <x:c r="J32" s="19"/>
       <x:c r="K32" s="3" t="str">
         <x:v>165 — Garde anonyme — salut de victoire
 10_VIE_DES_STAGES!E77</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="65.25" customHeight="1">
-      <x:c r="A33" s="16" t="n">
+      <x:c r="A33" s="18" t="n">
         <x:v>169</x:v>
       </x:c>
       <x:c r="B33" s="3" t="str">
@@ -1374,7 +1387,7 @@
       <x:c r="C33" s="3" t="str">
         <x:v>Transport de maintenance anonyme — roues</x:v>
       </x:c>
-      <x:c r="D33" s="16" t="n">
+      <x:c r="D33" s="18" t="n">
         <x:v>6</x:v>
       </x:c>
       <x:c r="E33" s="3" t="str">
@@ -1390,9 +1403,9 @@
         <x:v>Hydra fondé sur le manuel EA/Fox et le portrait original du jeu. Détails fins reconstruits. Masqué si Hydra combat.</x:v>
       </x:c>
       <x:c r="I33" s="3" t="str">
-        <x:v>Publication non vérifiée</x:v>
-      </x:c>
-      <x:c r="J33" s="17"/>
+        <x:v>Publié, lot contrôlé</x:v>
+      </x:c>
+      <x:c r="J33" s="19"/>
       <x:c r="K33" s="3" t="str">
         <x:v>169 — Transport de maintenance anonyme — roues
 10_VIE_DES_STAGES!A89:N91
@@ -1400,7 +1413,7 @@
       </x:c>
     </x:row>
     <x:row r="34" ht="87.75" customHeight="1">
-      <x:c r="A34" s="16" t="n">
+      <x:c r="A34" s="18" t="n">
         <x:v>169</x:v>
       </x:c>
       <x:c r="B34" s="3" t="str">
@@ -1409,7 +1422,7 @@
       <x:c r="C34" s="3" t="str">
         <x:v>Hydra — contrôle de la batterie dorsale</x:v>
       </x:c>
-      <x:c r="D34" s="16" t="n">
+      <x:c r="D34" s="18" t="n">
         <x:v>6</x:v>
       </x:c>
       <x:c r="E34" s="3" t="str">
@@ -1425,9 +1438,9 @@
         <x:v>Hydra fondé sur le manuel EA/Fox et le portrait original du jeu. Détails fins reconstruits. Masqué si Hydra combat.</x:v>
       </x:c>
       <x:c r="I34" s="3" t="str">
-        <x:v>Publication non vérifiée</x:v>
-      </x:c>
-      <x:c r="J34" s="17"/>
+        <x:v>Publié, lot contrôlé</x:v>
+      </x:c>
+      <x:c r="J34" s="19"/>
       <x:c r="K34" s="3" t="str">
         <x:v>169 — Hydra — contrôle de la batterie dorsale
 10_VIE_DES_STAGES!A90:N90
@@ -1436,7 +1449,7 @@
       </x:c>
     </x:row>
     <x:row r="35" ht="65.25" customHeight="1">
-      <x:c r="A35" s="16" t="n">
+      <x:c r="A35" s="18" t="n">
         <x:v>169</x:v>
       </x:c>
       <x:c r="B35" s="3" t="str">
@@ -1445,7 +1458,7 @@
       <x:c r="C35" s="3" t="str">
         <x:v>Balise de front originale — volet diagnostique</x:v>
       </x:c>
-      <x:c r="D35" s="16" t="n">
+      <x:c r="D35" s="18" t="n">
         <x:v>6</x:v>
       </x:c>
       <x:c r="E35" s="3" t="str">
@@ -1461,9 +1474,9 @@
         <x:v>Hydra fondé sur le manuel EA/Fox et le portrait original du jeu. Détails fins reconstruits. Masqué si Hydra combat.</x:v>
       </x:c>
       <x:c r="I35" s="3" t="str">
-        <x:v>Publication non vérifiée</x:v>
-      </x:c>
-      <x:c r="J35" s="17"/>
+        <x:v>Publié, lot contrôlé</x:v>
+      </x:c>
+      <x:c r="J35" s="19"/>
       <x:c r="K35" s="3" t="str">
         <x:v>169 — Balise de front originale — volet diagnostique
 10_VIE_DES_STAGES!A89:N91
@@ -1471,7 +1484,7 @@
       </x:c>
     </x:row>
     <x:row r="36" ht="48" customHeight="1">
-      <x:c r="A36" s="16" t="n">
+      <x:c r="A36" s="18" t="n">
         <x:v>173</x:v>
       </x:c>
       <x:c r="B36" s="3" t="str">
@@ -1480,7 +1493,7 @@
       <x:c r="C36" s="3" t="str">
         <x:v>Cloche de départ — frappe unique du battant</x:v>
       </x:c>
-      <x:c r="D36" s="16" t="n">
+      <x:c r="D36" s="18" t="n">
         <x:v>6</x:v>
       </x:c>
       <x:c r="E36" s="3" t="str">
@@ -1496,16 +1509,16 @@
         <x:v>Cloche liée au début de manche. La lanterne passive est remplacée pendant le geste. Architecture originale adaptée.</x:v>
       </x:c>
       <x:c r="I36" s="3" t="str">
-        <x:v>Publication non vérifiée</x:v>
-      </x:c>
-      <x:c r="J36" s="17"/>
+        <x:v>Publié, lot contrôlé</x:v>
+      </x:c>
+      <x:c r="J36" s="19"/>
       <x:c r="K36" s="3" t="str">
         <x:v>173 — Cloche de départ — frappe unique du battant
 10_VIE_DES_STAGES!E118</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="48" customHeight="1">
-      <x:c r="A37" s="16" t="n">
+      <x:c r="A37" s="18" t="n">
         <x:v>185</x:v>
       </x:c>
       <x:c r="B37" s="3" t="str">
@@ -1514,7 +1527,7 @@
       <x:c r="C37" s="3" t="str">
         <x:v>Arbitre anonyme — jugement de fin de manche</x:v>
       </x:c>
-      <x:c r="D37" s="16" t="n">
+      <x:c r="D37" s="18" t="n">
         <x:v>6</x:v>
       </x:c>
       <x:c r="E37" s="3" t="str">
@@ -1530,9 +1543,9 @@
         <x:v>Jugement d’un ancien anonyme en fin de manche. Aucun verdict narratif ou pouvoir canonique ajouté.</x:v>
       </x:c>
       <x:c r="I37" s="3" t="str">
-        <x:v>Publication non vérifiée</x:v>
-      </x:c>
-      <x:c r="J37" s="17"/>
+        <x:v>Publié, lot contrôlé</x:v>
+      </x:c>
+      <x:c r="J37" s="19"/>
       <x:c r="K37" s="3" t="str">
         <x:v>185 — Arbitre anonyme — jugement de fin de manche
 10_VIE_DES_STAGES!E166</x:v>
@@ -1541,7 +1554,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R58bd1a26d03940d0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4fe74ebc28634bf2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1642,30 +1655,30 @@
       <x:c r="G7" s="3"/>
     </x:row>
     <x:row r="8" ht="36" customHeight="1">
-      <x:c r="A8" s="13" t="str">
+      <x:c r="A8" s="15" t="str">
         <x:v>Scène</x:v>
       </x:c>
-      <x:c r="B8" s="13" t="str">
+      <x:c r="B8" s="15" t="str">
         <x:v>Sujet</x:v>
       </x:c>
-      <x:c r="C8" s="13" t="str">
+      <x:c r="C8" s="15" t="str">
         <x:v>Demande</x:v>
       </x:c>
-      <x:c r="D8" s="13" t="str">
+      <x:c r="D8" s="15" t="str">
         <x:v>État</x:v>
       </x:c>
-      <x:c r="E8" s="13" t="str">
+      <x:c r="E8" s="15" t="str">
         <x:v>Constat vérifié</x:v>
       </x:c>
-      <x:c r="F8" s="13" t="str">
+      <x:c r="F8" s="15" t="str">
         <x:v>Suite nécessaire</x:v>
       </x:c>
-      <x:c r="G8" s="13" t="str">
+      <x:c r="G8" s="15" t="str">
         <x:v>Source V54</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="48" customHeight="1">
-      <x:c r="A9" s="16" t="n">
+      <x:c r="A9" s="18" t="n">
         <x:v>126</x:v>
       </x:c>
       <x:c r="B9" s="3" t="str">
@@ -1690,7 +1703,7 @@
       </x:c>
     </x:row>
     <x:row r="10" ht="48" customHeight="1">
-      <x:c r="A10" s="16" t="n">
+      <x:c r="A10" s="18" t="n">
         <x:v>51</x:v>
       </x:c>
       <x:c r="B10" s="3" t="str">
@@ -1715,7 +1728,7 @@
       </x:c>
     </x:row>
     <x:row r="11" ht="48" customHeight="1">
-      <x:c r="A11" s="16" t="n">
+      <x:c r="A11" s="18" t="n">
         <x:v>130</x:v>
       </x:c>
       <x:c r="B11" s="3" t="str">
@@ -1740,7 +1753,7 @@
       </x:c>
     </x:row>
     <x:row r="12" ht="65.25" customHeight="1">
-      <x:c r="A12" s="16" t="n">
+      <x:c r="A12" s="18" t="n">
         <x:v>119</x:v>
       </x:c>
       <x:c r="B12" s="3" t="str">
@@ -1765,7 +1778,7 @@
       </x:c>
     </x:row>
     <x:row r="13" ht="48" customHeight="1">
-      <x:c r="A13" s="16" t="n">
+      <x:c r="A13" s="18" t="n">
         <x:v>146</x:v>
       </x:c>
       <x:c r="B13" s="3" t="str">
@@ -1788,7 +1801,7 @@
       </x:c>
     </x:row>
     <x:row r="14" ht="48" customHeight="1">
-      <x:c r="A14" s="16" t="n">
+      <x:c r="A14" s="18" t="n">
         <x:v>155</x:v>
       </x:c>
       <x:c r="B14" s="3" t="str">
@@ -1811,7 +1824,7 @@
       </x:c>
     </x:row>
     <x:row r="15" ht="48" customHeight="1">
-      <x:c r="A15" s="16" t="n">
+      <x:c r="A15" s="18" t="n">
         <x:v>156</x:v>
       </x:c>
       <x:c r="B15" s="3" t="str">
@@ -1834,7 +1847,7 @@
       </x:c>
     </x:row>
     <x:row r="16" ht="48" customHeight="1">
-      <x:c r="A16" s="16" t="n">
+      <x:c r="A16" s="18" t="n">
         <x:v>162</x:v>
       </x:c>
       <x:c r="B16" s="3" t="str">
@@ -1857,7 +1870,7 @@
       </x:c>
     </x:row>
     <x:row r="17" ht="48" customHeight="1">
-      <x:c r="A17" s="16" t="n">
+      <x:c r="A17" s="18" t="n">
         <x:v>168</x:v>
       </x:c>
       <x:c r="B17" s="3" t="str">
@@ -1880,7 +1893,7 @@
       </x:c>
     </x:row>
     <x:row r="18" ht="48" customHeight="1">
-      <x:c r="A18" s="16" t="n">
+      <x:c r="A18" s="18" t="n">
         <x:v>170</x:v>
       </x:c>
       <x:c r="B18" s="3" t="str">
@@ -1903,7 +1916,7 @@
       </x:c>
     </x:row>
     <x:row r="19" ht="48" customHeight="1">
-      <x:c r="A19" s="16" t="n">
+      <x:c r="A19" s="18" t="n">
         <x:v>171</x:v>
       </x:c>
       <x:c r="B19" s="3" t="str">
@@ -1926,7 +1939,7 @@
       </x:c>
     </x:row>
     <x:row r="20" ht="48" customHeight="1">
-      <x:c r="A20" s="16" t="n">
+      <x:c r="A20" s="18" t="n">
         <x:v>178</x:v>
       </x:c>
       <x:c r="B20" s="3" t="str">
@@ -1949,7 +1962,7 @@
       </x:c>
     </x:row>
     <x:row r="21" ht="48" customHeight="1">
-      <x:c r="A21" s="16" t="n">
+      <x:c r="A21" s="18" t="n">
         <x:v>179</x:v>
       </x:c>
       <x:c r="B21" s="3" t="str">
@@ -1972,7 +1985,7 @@
       </x:c>
     </x:row>
     <x:row r="22" ht="48" customHeight="1">
-      <x:c r="A22" s="16" t="n">
+      <x:c r="A22" s="18" t="n">
         <x:v>180</x:v>
       </x:c>
       <x:c r="B22" s="3" t="str">
@@ -1995,7 +2008,7 @@
       </x:c>
     </x:row>
     <x:row r="23" ht="48" customHeight="1">
-      <x:c r="A23" s="16"/>
+      <x:c r="A23" s="18"/>
       <x:c r="B23" s="3" t="str">
         <x:v>Autres demandes du V54</x:v>
       </x:c>
@@ -2016,7 +2029,7 @@
       </x:c>
     </x:row>
     <x:row r="24" ht="48" customHeight="1">
-      <x:c r="A24" s="16"/>
+      <x:c r="A24" s="18"/>
       <x:c r="B24" s="3" t="str">
         <x:v>Adaptations des nouvelles ambiances</x:v>
       </x:c>
@@ -2039,7 +2052,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd326aa2e030e4de1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc775f892131d4a32"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>